<commit_message>
Mise a jour du 03-09-2026 13:04:23.34
</commit_message>
<xml_diff>
--- a/contenu/Seconde.xlsx
+++ b/contenu/Seconde.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="14370" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,18 +19,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -407,7 +401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U178"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6"/>
   <cols>
     <col width="2.921875" customWidth="1" style="1" min="1" max="1"/>
@@ -567,8 +561,19 @@
       <c r="L2" s="3" t="n"/>
     </row>
     <row r="3" ht="43.75" customHeight="1" s="1">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
       <c r="C3" t="n">
         <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2.SF1.2</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -581,9 +586,20 @@
       <c r="O3" s="3" t="n"/>
     </row>
     <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
       <c r="C4" t="n">
         <v>3</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2.SF1.3</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Arrondir un nombre</t>
@@ -592,9 +608,20 @@
       <c r="F4" s="3" t="n"/>
     </row>
     <row r="5" ht="29.15" customHeight="1" s="1">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
       <c r="C5" t="n">
         <v>4</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2.SF1.4</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Utiliser les notions de multiple, diviseur</t>
@@ -619,9 +646,20 @@
       <c r="L5" s="3" t="n"/>
     </row>
     <row r="6" ht="29.15" customHeight="1" s="1">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
       <c r="C6" t="n">
         <v>5</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2.SF1.5</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Savoir raisonner en utilisant la parité</t>
@@ -653,6 +691,12 @@
       </c>
     </row>
     <row r="7" ht="29.15" customHeight="1" s="1">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
       <c r="I7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
     </row>
@@ -698,163 +742,6 @@
     <row r="21" ht="43.75" customHeight="1" s="1">
       <c r="F21" s="3" t="n"/>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -872,7 +759,8 @@
     <col width="11.07421875" customWidth="1" style="1" min="1" max="1"/>
     <col width="60" customWidth="1" style="1" min="2" max="2"/>
     <col width="2.69140625" customWidth="1" style="1" min="3" max="237"/>
-    <col width="11.07421875" customWidth="1" style="1" min="238" max="16384"/>
+    <col width="11.07421875" customWidth="1" style="1" min="238" max="238"/>
+    <col width="11.07421875" customWidth="1" style="1" min="239" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="59.15" customHeight="1" s="1">
@@ -1621,6 +1509,16 @@
       <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2.SF1.2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Encadrer un nombre</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1639,12 +1537,42 @@
       <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2.SF1.3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Arrondir un nombre</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2.SF1.4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Utiliser les notions de multiple, diviseur</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2.SF1.5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Savoir raisonner en utilisant la parité</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
@@ -2333,9 +2261,7 @@
   <dimension ref="A1:AQ16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <cols>
-    <col width="3.69140625" customWidth="1" style="1" min="2" max="16"/>
-    <col width="3.69140625" customWidth="1" style="1" min="17" max="17"/>
-    <col width="3.69140625" customWidth="1" style="1" min="18" max="43"/>
+    <col width="3.69140625" customWidth="1" style="1" min="2" max="43"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>